<commit_message>
test commit after merge
</commit_message>
<xml_diff>
--- a/EnvGen2.xlsx
+++ b/EnvGen2.xlsx
@@ -1325,7 +1325,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1443,7 +1443,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -54116,7 +54116,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>19</v>
@@ -54179,7 +54179,7 @@
       <c r="Q6" s="7"/>
       <c r="R6" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -54205,7 +54205,7 @@
       </c>
       <c r="R7" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -54229,7 +54229,7 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -54253,7 +54253,7 @@
       <c r="Q9" s="14"/>
       <c r="R9" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -54273,7 +54273,7 @@
       <c r="Q10" s="14"/>
       <c r="R10" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -54293,7 +54293,7 @@
       <c r="Q11" s="14"/>
       <c r="R11" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -54313,7 +54313,7 @@
       <c r="Q12" s="14"/>
       <c r="R12" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -54333,7 +54333,7 @@
       <c r="Q13" s="14"/>
       <c r="R13" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -54353,7 +54353,7 @@
       <c r="Q14" s="14"/>
       <c r="R14" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -54373,7 +54373,7 @@
       <c r="Q15" s="14"/>
       <c r="R15" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="14"/>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
@@ -54393,7 +54393,7 @@
       <c r="Q16" s="14"/>
       <c r="R16" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="14"/>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
@@ -54413,7 +54413,7 @@
       <c r="Q17" s="14"/>
       <c r="R17" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="14"/>
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
@@ -54433,7 +54433,7 @@
       <c r="Q18" s="14"/>
       <c r="R18" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
@@ -54453,7 +54453,7 @@
       <c r="Q19" s="14"/>
       <c r="R19" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -54473,7 +54473,7 @@
       <c r="Q20" s="14"/>
       <c r="R20" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="14"/>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
@@ -54493,7 +54493,7 @@
       <c r="Q21" s="14"/>
       <c r="R21" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="14"/>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -54513,7 +54513,7 @@
       <c r="Q22" s="14"/>
       <c r="R22" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="14"/>
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
@@ -54533,7 +54533,7 @@
       <c r="Q23" s="14"/>
       <c r="R23" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="14"/>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
@@ -54553,7 +54553,7 @@
       <c r="Q24" s="14"/>
       <c r="R24" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="14"/>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -54573,7 +54573,7 @@
       <c r="Q25" s="14"/>
       <c r="R25" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="14"/>
       <c r="B26" s="14"/>
       <c r="C26" s="14"/>
@@ -54593,7 +54593,7 @@
       <c r="Q26" s="14"/>
       <c r="R26" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="14"/>
       <c r="B27" s="14"/>
       <c r="C27" s="14"/>
@@ -54613,7 +54613,7 @@
       <c r="Q27" s="14"/>
       <c r="R27" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="14"/>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
@@ -54633,7 +54633,7 @@
       <c r="Q28" s="14"/>
       <c r="R28" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="14"/>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
@@ -54653,7 +54653,7 @@
       <c r="Q29" s="14"/>
       <c r="R29" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
       <c r="A30" s="14"/>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -54673,7 +54673,7 @@
       <c r="Q30" s="14"/>
       <c r="R30" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="14"/>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
@@ -54693,7 +54693,7 @@
       <c r="Q31" s="14"/>
       <c r="R31" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -54713,7 +54713,7 @@
       <c r="Q32" s="14"/>
       <c r="R32" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
       <c r="A33" s="14"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -54733,7 +54733,7 @@
       <c r="Q33" s="14"/>
       <c r="R33" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
       <c r="A34" s="14"/>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -54753,7 +54753,7 @@
       <c r="Q34" s="14"/>
       <c r="R34" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="19.5">
       <c r="A35" s="14"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -54773,7 +54773,7 @@
       <c r="Q35" s="14"/>
       <c r="R35" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
       <c r="A36" s="14"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
@@ -54793,7 +54793,7 @@
       <c r="Q36" s="14"/>
       <c r="R36" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="14"/>
@@ -54813,7 +54813,7 @@
       <c r="Q37" s="14"/>
       <c r="R37" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="15.75">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5">
       <c r="A38" s="14"/>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>

</xml_diff>